<commit_message>
feat(ai): support shorthand payment schedule 0 for immediate and N for days
</commit_message>
<xml_diff>
--- a/Ho So Du An/Yeu Cau Thanh Toan/đơn yêu cầu thanh toán - CÔNG TY TNHH CÔNG NGHỆ JINXUN VIỆT NAM - HD-20261013-001.xlsx
+++ b/Ho So Du An/Yeu Cau Thanh Toan/đơn yêu cầu thanh toán - CÔNG TY TNHH CÔNG NGHỆ JINXUN VIỆT NAM - HD-20261013-001.xlsx
@@ -1411,7 +1411,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A2:N31"/>
+  <dimension ref="A1:N31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15.6"/>
   <cols>
     <col width="5.796875" bestFit="1" customWidth="1" style="82" min="1" max="1"/>
@@ -1427,6 +1427,7 @@
     <col width="19.3984375" bestFit="1" customWidth="1" style="82" min="14" max="14"/>
   </cols>
   <sheetData>
+    <row r="1"/>
     <row r="2" ht="30.6" customHeight="1" s="82">
       <c r="B2" s="77" t="inlineStr">
         <is>
@@ -1809,7 +1810,7 @@
           <t>備註：
 ngay lập tức: Thanh toán 35% giá trị hợp đồng (282.654.114 VND - Hai trăm tám mươi hai triệu sáu trăm năm mươi tư nghìn một trăm mười bốn đồng chẵn.) Chưa thanh toán.
 01  第1期付款條件達成時：支付合約金額的 35% (282.654.114 VND，越南盾貳億捌仟貳佰陸拾伍萬肆仟壹佰壹拾肆整)。待支付。
-60 ngàu: Thanh toán 55% giá trị hợp đồng (444.170.751 VND - Bốn trăm bốn mươi tư triệu một trăm bảy mươi nghìn bảy trăm năm mươi mốt đồng chẵn.) Chưa thanh toán.
+60 ngày: Thanh toán 55% giá trị hợp đồng (444.170.751 VND - Bốn trăm bốn mươi tư triệu một trăm bảy mươi nghìn bảy trăm năm mươi mốt đồng chẵn.) Chưa thanh toán.
 02  第2期付款條件達成時：支付合約金額的 55% (444.170.751 VND，越南盾肆億肆仟肆佰壹拾柒萬零柒佰伍拾壹整)。待支付。
 kể từ ngày ký biên bản nghiệm thu bàn giao (FAC), thời hạn thanh toán T/T 60 ngày: Thanh toán 10% giá trị hợp đồng (80.758.318 VND - Tám mươi triệu bảy trăm năm mươi tám nghìn ba trăm mười tám đồng chẵn.) Chưa thanh toán.
 03  簽約完成時：支付合約金額的 10% (80.758.318 VND，越南盾捌仟零柒拾伍萬捌仟參佰壹拾捌整)。待支付。

</xml_diff>

<commit_message>
feat(quotation): add eco prime quotation generator
</commit_message>
<xml_diff>
--- a/Ho So Du An/Yeu Cau Thanh Toan/đơn yêu cầu thanh toán - CÔNG TY TNHH CÔNG NGHỆ JINXUN VIỆT NAM - HD-20261013-001.xlsx
+++ b/Ho So Du An/Yeu Cau Thanh Toan/đơn yêu cầu thanh toán - CÔNG TY TNHH CÔNG NGHỆ JINXUN VIỆT NAM - HD-20261013-001.xlsx
@@ -1411,7 +1411,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:N31"/>
+  <dimension ref="A2:N31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15.6"/>
   <cols>
     <col width="5.796875" bestFit="1" customWidth="1" style="82" min="1" max="1"/>
@@ -1427,7 +1427,6 @@
     <col width="19.3984375" bestFit="1" customWidth="1" style="82" min="14" max="14"/>
   </cols>
   <sheetData>
-    <row r="1"/>
     <row r="2" ht="30.6" customHeight="1" s="82">
       <c r="B2" s="77" t="inlineStr">
         <is>
@@ -1501,7 +1500,7 @@
       </c>
       <c r="H9" s="70" t="inlineStr">
         <is>
-          <t>HMV16102026-001-SYTT</t>
+          <t>HMV17102026-001-SYTT</t>
         </is>
       </c>
       <c r="K9" s="83" t="n"/>
@@ -1525,7 +1524,7 @@
         </is>
       </c>
       <c r="I10" s="46" t="n">
-        <v>46311</v>
+        <v>46312</v>
       </c>
       <c r="K10" s="83" t="n"/>
     </row>
@@ -1553,7 +1552,11 @@
 Ngày đến hạn thanh toán:</t>
         </is>
       </c>
-      <c r="C12" s="73" t="inlineStr"/>
+      <c r="C12" s="73" t="inlineStr">
+        <is>
+          <t>25/10/2026</t>
+        </is>
+      </c>
       <c r="F12" s="75" t="inlineStr">
         <is>
           <t>付 款 方 式：
@@ -1633,7 +1636,8 @@
       <c r="B15" s="39" t="inlineStr">
         <is>
           <t>請款 / Thanh toán Đợt 1: 35%
-合約 / Hợp đồng：HD-20261013-001</t>
+合約 / Hợp đồng：HD-20261013-001
+發票 / Hóa đơn：HD-TEST-001</t>
         </is>
       </c>
       <c r="C15" s="85" t="inlineStr">
@@ -1808,9 +1812,9 @@
       <c r="B23" s="97" t="inlineStr">
         <is>
           <t>備註：
-ngay lập tức: Thanh toán 35% giá trị hợp đồng (282.654.114 VND - Hai trăm tám mươi hai triệu sáu trăm năm mươi tư nghìn một trăm mười bốn đồng chẵn.) Chưa thanh toán.
-01  第1期付款條件達成時：支付合約金額的 35% (282.654.114 VND，越南盾貳億捌仟貳佰陸拾伍萬肆仟壹佰壹拾肆整)。待支付。
-60 ngày: Thanh toán 55% giá trị hợp đồng (444.170.751 VND - Bốn trăm bốn mươi tư triệu một trăm bảy mươi nghìn bảy trăm năm mươi mốt đồng chẵn.) Chưa thanh toán.
+ngay lập tức: Thanh toán 35% giá trị hợp đồng (282.654.114 VND - Hai trăm tám mươi hai triệu sáu trăm năm mươi tư nghìn một trăm mười bốn đồng chẵn.) Hạn thanh toán: 25/10/2026. Hóa đơn: HD-TEST-001. Chưa thanh toán.
+01  第1期付款條件達成時：支付合約金額的 35% (282.654.114 VND，越南盾貳億捌仟貳佰陸拾伍萬肆仟壹佰壹拾肆整)。 付款到期日：25/10/2026。 發票編號：HD-TEST-001。待支付。
+thời hạn thanh toán T/T 60 ngày: Thanh toán 55% giá trị hợp đồng (444.170.751 VND - Bốn trăm bốn mươi tư triệu một trăm bảy mươi nghìn bảy trăm năm mươi mốt đồng chẵn.) Chưa thanh toán.
 02  第2期付款條件達成時：支付合約金額的 55% (444.170.751 VND，越南盾肆億肆仟肆佰壹拾柒萬零柒佰伍拾壹整)。待支付。
 kể từ ngày ký biên bản nghiệm thu bàn giao (FAC), thời hạn thanh toán T/T 60 ngày: Thanh toán 10% giá trị hợp đồng (80.758.318 VND - Tám mươi triệu bảy trăm năm mươi tám nghìn ba trăm mười tám đồng chẵn.) Chưa thanh toán.
 03  簽約完成時：支付合約金額的 10% (80.758.318 VND，越南盾捌仟零柒拾伍萬捌仟參佰壹拾捌整)。待支付。

</xml_diff>